<commit_message>
feat: add possibility for player to type in the text area and send a message
</commit_message>
<xml_diff>
--- a/maeve_dialogue.xlsx
+++ b/maeve_dialogue.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Binbin\Documents\maeve----lost-signal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{38F3F78C-F9FB-4F3A-86FD-F5D79DCDD5DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38E23CE9-D824-4C26-A0BC-4BB8079BB40F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21840" xr2:uid="{F3A416B8-D169-4D51-BEC7-403A75AE62E5}"/>
+    <workbookView xWindow="4065" yWindow="4710" windowWidth="38700" windowHeight="15885" xr2:uid="{F3A416B8-D169-4D51-BEC7-403A75AE62E5}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Bonjour?</t>
   </si>
@@ -80,45 +80,18 @@
     <t>Si c'est une blague c'est vraiment pas drole.</t>
   </si>
   <si>
-    <t xml:space="preserve">Ok calmez vous </t>
-  </si>
-  <si>
     <t>J'ai essayé des dizaines de numéros mais aucun message ne s'envoie a part sur ce numéro apparemment…</t>
   </si>
   <si>
-    <t>Je vais vous aider</t>
-  </si>
-  <si>
     <t>Je vous promet que non!</t>
   </si>
   <si>
-    <t>Vraiment?</t>
-  </si>
-  <si>
-    <t>Oui pardon… Vous avez raison…</t>
-  </si>
-  <si>
     <t>Je comprends que ca puisse laisser cette impression  mais c'est vraiment pas le cas!</t>
   </si>
   <si>
-    <t xml:space="preserve">Enfin un truc positif dans cette journée pourrie! </t>
-  </si>
-  <si>
-    <t>C'est pas évident mais il faut que je garde la tête froide si je veux pouvoir sortir d'ici</t>
-  </si>
-  <si>
     <t>Je vous en supplie, restez avec moi! J'ai vraiment besoin d'aide!</t>
   </si>
   <si>
-    <t>Merci merci merci</t>
-  </si>
-  <si>
-    <t>Merci! Avoir quelqu'un avec qui partager ce qu'il se passe devrait aider.</t>
-  </si>
-  <si>
-    <t>Mouais je suis pas toujours pas super convaincu…</t>
-  </si>
-  <si>
     <t>Pour l'instant</t>
   </si>
   <si>
@@ -126,6 +99,39 @@
   </si>
   <si>
     <t>Ok ok je sais pas quoi penser mais je vais rester,,,</t>
+  </si>
+  <si>
+    <t>Wow… Bon je sais pas trop comment mais je veux bien essayer de vous aider.</t>
+  </si>
+  <si>
+    <t>Franchement, au point ou j'en suis c'est déjà énorme!</t>
+  </si>
+  <si>
+    <t>Ca fait au moins un truc de positif dans cette journée pourrie</t>
+  </si>
+  <si>
+    <t>Mouais... je suis pas super convaincu…</t>
+  </si>
+  <si>
+    <t>Rien que le fait de pouvoir parler avec quelqu'un c'est déjà rassurant!</t>
+  </si>
+  <si>
+    <t>Je suis pas sur de pouvoir aider la! C'est pas que je vous crois pas mais je vois pas trop ce que je peux faire…</t>
+  </si>
+  <si>
+    <t>Etre la c'est un bon début</t>
+  </si>
+  <si>
+    <t>Je dois garder la tête froide et éviter de devenir folle ou de me mettre en boule et pleurer…</t>
+  </si>
+  <si>
+    <t>Je suis désolé de vous demander de m'aider mais j'ai vraiment pas d'autre choix!</t>
+  </si>
+  <si>
+    <t>Je m'appelle Maeve</t>
+  </si>
+  <si>
+    <t>Bon si on est emmené à rester ensemble un moment on peut au moins présenter</t>
   </si>
 </sst>
 </file>
@@ -175,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -187,9 +193,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -529,7 +532,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0281E8E-1DAF-4EA9-88E0-6092A0CF41BF}">
-  <dimension ref="A1:AK15"/>
+  <dimension ref="A1:AK17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="16" width="11.42578125" style="1"/>
@@ -590,7 +593,7 @@
     </row>
     <row r="8" spans="18:21" ht="30" x14ac:dyDescent="0.25">
       <c r="T8" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="18:21" ht="30" x14ac:dyDescent="0.25">
@@ -598,68 +601,78 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="18:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="18:21" ht="30" x14ac:dyDescent="0.25">
       <c r="R10" s="4" t="s">
         <v>12</v>
       </c>
       <c r="S10" s="4"/>
       <c r="T10" s="3" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="U10" s="3" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="18:21" x14ac:dyDescent="0.25">
       <c r="R11" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="S11" s="5"/>
       <c r="T11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="U11" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="18:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="R12" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="S12" s="5"/>
+      <c r="T12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="U12" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="18:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="R13" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="S13" s="5"/>
+      <c r="T13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U13" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="18:21" x14ac:dyDescent="0.25">
+      <c r="R14" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="S14" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="18:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="R15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="S15" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="U11" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="18:21" ht="30" x14ac:dyDescent="0.25">
-      <c r="R12" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="S12" s="6"/>
-      <c r="T12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="U12" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="18:21" ht="30" x14ac:dyDescent="0.25">
-      <c r="R13" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="S13" s="6"/>
-      <c r="T13" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="U13" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="18:21" ht="30" x14ac:dyDescent="0.25">
-      <c r="R14" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="S14" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="15" spans="18:21" ht="30" x14ac:dyDescent="0.25">
-      <c r="R15" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="S15" s="1" t="s">
-        <v>26</v>
+    </row>
+    <row r="16" spans="18:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="T16" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="20:20" x14ac:dyDescent="0.25">
+      <c r="T17" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>